<commit_message>
Added fitting procedure for orthogonal datasets
</commit_message>
<xml_diff>
--- a/Sheets/BrShift.xlsx
+++ b/Sheets/BrShift.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11010"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38646499-627A-8C44-B2FE-C085E8D87E74}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C531B5B-C82B-C14E-AFCB-1FB651421132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="1460" windowWidth="27240" windowHeight="16040" xr2:uid="{85812D83-8DEC-B647-9A33-A6CE083631F3}"/>
   </bookViews>
@@ -500,8 +500,7 @@
     </row>
     <row r="6" spans="3:14" x14ac:dyDescent="0.2">
       <c r="C6" s="1">
-        <f>74.7989-74.7089</f>
-        <v>9.0000000000003411E-2</v>
+        <v>0.15</v>
       </c>
       <c r="D6">
         <f>SQRT(0.000908769^2+0.00167659^2)</f>
@@ -512,7 +511,7 @@
       </c>
       <c r="F6">
         <f>E6*C6</f>
-        <v>1.6470000000000624</v>
+        <v>2.7450000000000001</v>
       </c>
       <c r="G6">
         <f>D6*E6</f>
@@ -520,7 +519,7 @@
       </c>
       <c r="H6">
         <f>F6+$D$2</f>
-        <v>0.90500000000006242</v>
+        <v>2.0030000000000001</v>
       </c>
       <c r="I6">
         <f>SQRT($E$2^2+G6^2)</f>

</xml_diff>